<commit_message>
feat: rediseno UI dashboard + fix 403 health-data + QA mobile
- Rediseno completo del dashboard (sidebar dark, glassmorphism login,
  cards mejoradas, graficos con gradientes, responsive)
- Sidebar sticky para que no se mueva al hacer scroll
- Navegacion de cards de pacientes a ficha individual
- Fix bug 403 en endpoint /health-data (comparacion user_id vs patient_id)
- Tests Playwright dashboard (8 tests) + mobile (10 tests)
- Scripts de grabacion de demo y actualizacion de PPTX
- Reportes QA actualizados (52 tests)
</commit_message>
<xml_diff>
--- a/qa/Guion_de_Pruebas_MoodIoT.xlsx
+++ b/qa/Guion_de_Pruebas_MoodIoT.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidences" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$4:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tests'!$A$4:$L$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -695,7 +695,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>52</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -830,13 +830,13 @@
     </row>
     <row r="3">
       <c r="J3" s="13" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="K3" s="13" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -3575,8 +3575,651 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-01</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>Ecran de login de l'application mobile</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F47" s="14" t="inlineStr">
+        <is>
+          <t>Preview mobile accessible, backend demarre</t>
+        </is>
+      </c>
+      <c r="G47" s="14" t="inlineStr">
+        <is>
+          <t>1. Ouvrir l'application mobile
+2. Verifier la presence du formulaire de connexion
+3. Verifier les champs email et mot de passe</t>
+        </is>
+      </c>
+      <c r="H47" s="14" t="inlineStr">
+        <is>
+          <t>Formulaire de login affiche avec logo Mood-IoT et champs de saisie</t>
+        </is>
+      </c>
+      <c r="I47" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J47" s="14" t="inlineStr">
+        <is>
+          <t>Interface conforme aux specifications</t>
+        </is>
+      </c>
+      <c r="K47" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L47" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_01_login.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-02</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Connexion patient avec JWT (spinner)</t>
+        </is>
+      </c>
+      <c r="E48" s="18" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr">
+        <is>
+          <t>Identifiants patient valides (sophie.dupont@email.fr)</t>
+        </is>
+      </c>
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>1. Saisir email et mot de passe du patient
+2. Cliquer sur SE CONNECTER
+3. Verifier le spinner de chargement
+4. Verifier la requete POST /auth/login dans la console</t>
+        </is>
+      </c>
+      <c r="H48" s="17" t="inlineStr">
+        <is>
+          <t>Spinner affiche, requete HTTP envoyee, token JWT recu</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J48" s="17" t="inlineStr">
+        <is>
+          <t>Token JWT stocke en memoire pour les requetes suivantes</t>
+        </is>
+      </c>
+      <c r="K48" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L48" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_02_login_loading.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-03</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>Accueil patient apres authentification</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F49" s="14" t="inlineStr">
+        <is>
+          <t>Patient authentifie</t>
+        </is>
+      </c>
+      <c r="G49" s="14" t="inlineStr">
+        <is>
+          <t>1. Verifier l'ecran d'accueil apres login
+2. Verifier le message de bienvenue avec le nom du patient
+3. Verifier les statistiques vides avant synchronisation</t>
+        </is>
+      </c>
+      <c r="H49" s="14" t="inlineStr">
+        <is>
+          <t>Ecran principal affiche avec 'Bonjour, Sophie' et stats a '--'</t>
+        </is>
+      </c>
+      <c r="I49" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J49" s="14" t="inlineStr">
+        <is>
+          <t>Nom du patient recupere depuis la reponse du backend</t>
+        </is>
+      </c>
+      <c r="K49" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L49" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_03_accueil.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-04</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Synchronisation automatique Health Connect</t>
+        </is>
+      </c>
+      <c r="E50" s="18" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>Patient connecte, Health Connect avec donnees</t>
+        </is>
+      </c>
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>1. Observer la synchronisation automatique apres login
+2. Verifier la lecture Health Connect (Steps, HeartRate, SleepSession)
+3. Verifier le spinner de synchronisation</t>
+        </is>
+      </c>
+      <c r="H50" s="17" t="inlineStr">
+        <is>
+          <t>Lecture automatique des capteurs et envoi au backend lance</t>
+        </is>
+      </c>
+      <c r="I50" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J50" s="17" t="inlineStr">
+        <is>
+          <t>Sync automatique 1 seconde apres le login</t>
+        </is>
+      </c>
+      <c r="K50" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L50" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_04_sync_loading.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-05</t>
+        </is>
+      </c>
+      <c r="D51" s="14" t="inlineStr">
+        <is>
+          <t>Donnees synchronisees avec succes (badge vert)</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F51" s="14" t="inlineStr">
+        <is>
+          <t>Synchronisation en cours</t>
+        </is>
+      </c>
+      <c r="G51" s="14" t="inlineStr">
+        <is>
+          <t>1. Attendre la fin de la synchronisation
+2. Verifier le badge vert 'Synchronise a HH:MM'
+3. Verifier les valeurs PAS, BPM, SOMMEIL affichees
+4. Verifier la reponse du serveur dans la console</t>
+        </is>
+      </c>
+      <c r="H51" s="14" t="inlineStr">
+        <is>
+          <t>Badge vert, donnees affichees, reponse upserted:true dans la console</t>
+        </is>
+      </c>
+      <c r="I51" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J51" s="14" t="inlineStr">
+        <is>
+          <t>Console affiche le payload envoye et la reponse du serveur</t>
+        </is>
+      </c>
+      <c r="K51" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L51" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_05_sync_ok.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-06</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Re-synchronisation UPSERT (pas de doublon)</t>
+        </is>
+      </c>
+      <c r="E52" s="18" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
+        <is>
+          <t>Premiere synchronisation effectuee</t>
+        </is>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>1. Cliquer sur SYNCHRONISER une deuxieme fois
+2. Verifier que les nouvelles donnees sont envoyees
+3. Verifier dans la console que l'UPSERT met a jour sans creer de doublon</t>
+        </is>
+      </c>
+      <c r="H52" s="17" t="inlineStr">
+        <is>
+          <t>Donnees mises a jour, une seule ligne par (patient_id, date) en BD</t>
+        </is>
+      </c>
+      <c r="I52" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J52" s="17" t="inlineStr">
+        <is>
+          <t>UPSERT ON CONFLICT (patient_id, date) DO UPDATE</t>
+        </is>
+      </c>
+      <c r="K52" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L52" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_06_resync.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-07</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>Verification donnees dans PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>Synchronisation effectuee</t>
+        </is>
+      </c>
+      <c r="G53" s="14" t="inlineStr">
+        <is>
+          <t>1. Executer SELECT sur daily_aggregates pour le patient
+2. Verifier heart_rate_avg, step_count, sleep_duration_min
+3. Verifier source_platform = android_health_connect
+4. Verifier synced_at horodate</t>
+        </is>
+      </c>
+      <c r="H53" s="14" t="inlineStr">
+        <is>
+          <t>Donnees presentes dans PostgreSQL avec tous les champs remplis</t>
+        </is>
+      </c>
+      <c r="I53" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J53" s="14" t="inlineStr">
+        <is>
+          <t>Champ source_platform permet de distinguer Android vs iOS</t>
+        </is>
+      </c>
+      <c r="K53" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L53" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_07_db_check.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-08</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Batch sync de 3 jours offline</t>
+        </is>
+      </c>
+      <c r="E54" s="18" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>Token JWT valide, endpoint batch disponible</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>1. POST /patients/{id}/health-data/batch avec 3 jours de donnees
+2. Verifier la reponse synced_count = 3
+3. Verifier les 3 enregistrements en BD</t>
+        </is>
+      </c>
+      <c r="H54" s="17" t="inlineStr">
+        <is>
+          <t>3 jours synchronises en une seule requete, reponse synced_count:3</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J54" s="17" t="inlineStr">
+        <is>
+          <t>Simule un patient qui n'a pas ouvert l'app pendant 3 jours</t>
+        </is>
+      </c>
+      <c r="K54" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L54" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_08_batch_api.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-09</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>Verification batch dans PostgreSQL</t>
+        </is>
+      </c>
+      <c r="E55" s="15" t="inlineStr">
+        <is>
+          <t>Haute</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>Batch sync effectue</t>
+        </is>
+      </c>
+      <c r="G55" s="14" t="inlineStr">
+        <is>
+          <t>1. SELECT COUNT(*) FROM daily_aggregates pour le patient
+2. Verifier que tous les jours sont presents
+3. Verifier l'absence de doublons</t>
+        </is>
+      </c>
+      <c r="H55" s="14" t="inlineStr">
+        <is>
+          <t>7 enregistrements uniques dans daily_aggregates</t>
+        </is>
+      </c>
+      <c r="I55" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J55" s="14" t="inlineStr">
+        <is>
+          <t>Chaque jour = une seule ligne grace a l'UPSERT</t>
+        </is>
+      </c>
+      <c r="K55" s="14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L55" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_09_db_batch.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-10</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Deconnexion de l'application mobile</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
+        <is>
+          <t>Patient connecte</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>1. Cliquer sur Deconnexion
+2. Verifier la suppression du token JWT
+3. Verifier le retour a l'ecran de login</t>
+        </is>
+      </c>
+      <c r="H56" s="17" t="inlineStr">
+        <is>
+          <t>Token supprime, retour a l'ecran de connexion</t>
+        </is>
+      </c>
+      <c r="I56" s="16" t="inlineStr">
+        <is>
+          <t>Reussi</t>
+        </is>
+      </c>
+      <c r="J56" s="17" t="inlineStr">
+        <is>
+          <t>Aucune donnee sensible accessible apres deconnexion</t>
+        </is>
+      </c>
+      <c r="K56" s="17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L56" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_10_logout.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L46"/>
+  <autoFilter ref="A4:L56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3588,7 +4231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3613,7 +4256,7 @@
         </is>
       </c>
       <c r="B3" s="21" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4">
@@ -3623,7 +4266,7 @@
         </is>
       </c>
       <c r="B4" s="22" t="n">
-        <v>42</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -3931,23 +4574,49 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="24" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>UC 10</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>App Mobile Health Connect</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="B22" s="25" t="n"/>
-      <c r="C22" s="26" t="n">
-        <v>42</v>
-      </c>
-      <c r="D22" s="26" t="n">
-        <v>42</v>
-      </c>
-      <c r="E22" s="26" t="n">
+      <c r="B23" s="25" t="n"/>
+      <c r="C23" s="26" t="n">
+        <v>52</v>
+      </c>
+      <c r="D23" s="26" t="n">
+        <v>52</v>
+      </c>
+      <c r="E23" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="27" t="inlineStr">
+      <c r="F23" s="27" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
@@ -3956,7 +4625,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3969,7 +4638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4715,6 +5384,176 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-01</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>Ecran de login de l'application mobile</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_01_login.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-02</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>Connexion patient avec JWT (spinner)</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_02_login_loading.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-03</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>Accueil patient apres authentification</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_03_accueil.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-04</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Synchronisation automatique Health Connect</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_04_sync_loading.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-05</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>Donnees synchronisees avec succes (badge vert)</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_05_sync_ok.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-06</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>Re-synchronisation UPSERT (pas de doublon)</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_06_resync.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-07</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>Verification donnees dans PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_07_db_check.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-08</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>Batch sync de 3 jours offline</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_08_batch_api.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>TC-UC10-09</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Verification batch dans PostgreSQL</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>sc_mob_09_db_batch.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>TC-UC10-10</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>Deconnexion de l'application mobile</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>sc_mob_10_logout.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>